<commit_message>
chore(audit): mark BUG-057/082/087/101/103/109/116/138/139 Fixed in R6 tracker
Writes per-bug Developer comments + Fixed in build=2026-10-14 for
every bug closed this session. SHAs link back to the fix commits.
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -9714,18 +9714,18 @@
       </c>
       <c r="Z58" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA58" s="15" t="n"/>
       <c r="AB58" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: FEDEX label vocab needs full form↔registry unification across both directions.</t>
+          <t>Fixed on dev (839f1ef8): FEDEX order form + per-carrier editor modals now read labelFormatsForCarrier() (DB registry); FEDEX added to the bootstrap list to mirror V120 seed.</t>
         </is>
       </c>
       <c r="AC58" s="15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -13055,16 +13055,20 @@
       </c>
       <c r="Z83" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA83" s="15" t="n"/>
       <c r="AB83" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Address book field validation needs yup schema wiring; defer.</t>
-        </is>
-      </c>
-      <c r="AC83" s="15" t="n"/>
+          <t>Fixed on dev (9796ed31): Address book now runs the shared validatePhoneForCountry / validateEmail / validateZip / STATE_CODE_SETS checks before POST.</t>
+        </is>
+      </c>
+      <c r="AC83" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -13730,16 +13734,20 @@
       </c>
       <c r="Z88" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA88" s="15" t="n"/>
       <c r="AB88" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Carrier Limits uses plain &lt;table&gt;, not AdvancedDataTable; needs grid migration.</t>
-        </is>
-      </c>
-      <c r="AC88" s="15" t="n"/>
+          <t>Fixed on dev (5088d31d): Templates got pinnedByDefault:'end' on actions column (BUG-025 mechanism). Carrier Limits uses sticky right:0 on &lt;th&gt;/&lt;td&gt; since it's a plain &lt;table&gt;.</t>
+        </is>
+      </c>
+      <c r="AC88" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
@@ -15604,16 +15612,20 @@
       </c>
       <c r="Z102" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA102" s="15" t="n"/>
       <c r="AB102" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Cutoff rules warehouse-id → warehouse-code picker.</t>
-        </is>
-      </c>
-      <c r="AC102" s="15" t="n"/>
+          <t>Fixed on dev (a8af5b2a): Cutoff rules grid shows warehouse code (loaded warehouses map); add-row swaps number input for dropdown.</t>
+        </is>
+      </c>
+      <c r="AC102" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
@@ -15869,16 +15881,20 @@
       </c>
       <c r="Z104" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA104" s="15" t="n"/>
       <c r="AB104" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Pickup form validation (window order, past date, 0 pkgs, phone shape).</t>
-        </is>
-      </c>
-      <c r="AC104" s="15" t="n"/>
+          <t>Fixed on dev (a8af5b2a): PickupsEodPage.runPickup rejects past date, inverted times, &lt;3-digit phone, bad postal, 0 packages BEFORE POST /pickups.</t>
+        </is>
+      </c>
+      <c r="AC104" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
@@ -16676,16 +16692,20 @@
       </c>
       <c r="Z110" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA110" s="15" t="n"/>
       <c r="AB110" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Templates Preview renders order's packing-slip not template; needs render path by template id.</t>
-        </is>
-      </c>
-      <c r="AC110" s="15" t="n"/>
+          <t>Fixed on dev (0fad4a45): Added renderWithTemplate(orderNo, templateId); controller ?templateId query param; FE passes previewContext.id so Preview renders THIS template.</t>
+        </is>
+      </c>
+      <c r="AC110" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -17626,16 +17646,20 @@
       </c>
       <c r="Z117" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA117" s="15" t="n"/>
       <c r="AB117" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Printer routing popover clipped by grid overflow; needs portal.</t>
-        </is>
-      </c>
-      <c r="AC117" s="15" t="n"/>
+          <t>Fixed on dev (fb113431): CellPopover createPortal'd to document.body with position:fixed, re-measured on scroll/resize; grid overflow no longer clips.</t>
+        </is>
+      </c>
+      <c r="AC117" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -20579,16 +20603,20 @@
       </c>
       <c r="Z139" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA139" s="15" t="n"/>
       <c r="AB139" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Draft resume keeps staged carrier account but not creds; needs explicit "credentials required" guard on Summary READY.</t>
-        </is>
-      </c>
-      <c r="AC139" s="15" t="n"/>
+          <t>Fixed on dev (a8af5b2a): carriersStepComplete requires every staged draft to carry non-blank clientId AND clientSecret.</t>
+        </is>
+      </c>
+      <c r="AC139" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -20712,16 +20740,20 @@
       </c>
       <c r="Z140" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA140" s="15" t="n"/>
       <c r="AB140" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Add Client always resumes last draft; needs Discard-draft action.</t>
-        </is>
-      </c>
-      <c r="AC140" s="15" t="n"/>
+          <t>Fixed on dev (a8af5b2a): + Add Client shows 'Discard draft' button when a persisted draft exists; clears the localStorage key + reloads to seed every field blank.</t>
+        </is>
+      </c>
+      <c r="AC140" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): mark BUG-135 Fixed in R6 tracker
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -20201,16 +20201,20 @@
       </c>
       <c r="Z136" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA136" s="15" t="n"/>
       <c r="AB136" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Alerts History tenant/order; needs alert-emission plumbing.</t>
-        </is>
-      </c>
-      <c r="AC136" s="15" t="n"/>
+          <t>Fixed on dev (d5f6d288): rollbackSuccessfulPiecesSera overload threads orderNo (parseLongSafe(referenceNumber)) + tenantCode (departmentNumber per PR #543) into the three SERA MPS rollback alerts; Alerts History Tenant/Order columns populated for them.</t>
+        </is>
+      </c>
+      <c r="AC136" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): mark R6+1 fixes for 2026-10-15 session
Extends 12 bug rows with the afeb4111 + e17bf946 commits:
BUG-022/046/061/075/087/089/110/118/119/121/125/134. Prior-round
comments preserved on their own line so audit history stays
single-cell.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bugs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Screens" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Flows" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Test data" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="_ledger" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screens" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flows" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test data" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ledger" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bugs'!$A$1:$AC$149</definedName>
@@ -5134,12 +5134,13 @@
       <c r="AA23" s="15" t="n"/>
       <c r="AB23" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (a601e4aa): Delivery log recipient filter now escapes % _ and query uses ESCAPE "\\".</t>
+          <t>Fixed on dev (a601e4aa): Delivery log recipient filter now escapes % _ and query uses ESCAPE "\\".
+R6+1 (afeb4111+e17bf946, 2026-10-15): Spread ESCAPE '\' + escapeLike() to WarehouseRepository, AdminUserService (Criteria API) and AuditLogRepositoryCustomImpl. Delivery-log fix (a601e4aa) now matches every other search path.</t>
         </is>
       </c>
       <c r="AC23" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8274,12 +8275,13 @@
       <c r="AA47" s="15" t="n"/>
       <c r="AB47" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (bf6e96b8): Warehouse Country swaps the free-text ISO-2 input for the shared CountrySelect used by /orders/new + address book + client wizard.</t>
+          <t>Fixed on dev (bf6e96b8): Warehouse Country swaps the free-text ISO-2 input for the shared CountrySelect used by /orders/new + address book + client wizard.
+R6+1 (e17bf946, 2026-10-15): _countryData.ts sources from utils/countries.ts; CountrySelect now exposes the full 250-country list. Address book dialog switched to CountrySelect so warehouse / client / address book agree.</t>
         </is>
       </c>
       <c r="AC47" s="15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -10261,12 +10263,13 @@
       <c r="AA62" s="15" t="n"/>
       <c r="AB62" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (cb9e4ed5): SystemChannelSection scrubbed TENANT_CHANNEL_NOT_ENABLED raw code; "tenant" -&gt; "client".</t>
+          <t>Fixed on dev (cb9e4ed5): SystemChannelSection scrubbed TENANT_CHANNEL_NOT_ENABLED raw code; "tenant" -&gt; "client".
+R6+1 (afeb4111+e17bf946, 2026-10-15): Scrubbed internal copy on SystemSettings specs (backend), workspaceRoutes descriptions, Carrier Accounts, Code Maps, Cutoffs &amp; Holidays, External Systems, SystemSettingsPage deployment banner, DTC Scheduler 'Last changed by V&lt;n&gt;', Carrier Limits resolver blurb.</t>
         </is>
       </c>
       <c r="AC62" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -12100,12 +12103,13 @@
       <c r="AA76" s="15" t="n"/>
       <c r="AB76" s="15" t="inlineStr">
         <is>
-          <t>Fix landed earlier this session: Importer/Broker in-app confirm shipped as 15ab13b8 earlier.</t>
+          <t>Fix landed earlier this session: Importer/Broker in-app confirm shipped as 15ab13b8 earlier.
+R6+1 (e17bf946, 2026-10-15): CustomFieldsPage.del() swapped window.confirm for notify.confirm (title + danger + confirmLabel). Matches Importer/Broker in-app pattern.</t>
         </is>
       </c>
       <c r="AC76" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -13740,12 +13744,13 @@
       <c r="AA88" s="15" t="n"/>
       <c r="AB88" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (5088d31d): Templates got pinnedByDefault:'end' on actions column (BUG-025 mechanism). Carrier Limits uses sticky right:0 on &lt;th&gt;/&lt;td&gt; since it's a plain &lt;table&gt;.</t>
+          <t>Fixed on dev (5088d31d): Templates got pinnedByDefault:'end' on actions column (BUG-025 mechanism). Carrier Limits uses sticky right:0 on &lt;th&gt;/&lt;td&gt; since it's a plain &lt;table&gt;.
+R6+1 (e17bf946, 2026-10-15): CarrierShippingLimitsPage table now uses border-separate + border-spacing-0 so Chrome's position:sticky on &lt;th&gt;/&lt;td&gt; actually sticks Actions at narrow viewports.</t>
         </is>
       </c>
       <c r="AC88" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -14006,12 +14011,13 @@
       <c r="AA90" s="15" t="n"/>
       <c r="AB90" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (6754690c): Allow branded packaging toggle hidden entirely for Ground-family services + inline amber note.</t>
+          <t>Fixed on dev (6754690c): Allow branded packaging toggle hidden entirely for Ground-family services + inline amber note.
+R6+1 (V161 afeb4111, 2026-10-15): V161 re-applies V30's branded_packaging_allowed=false for UPS/FEDEX/USPS ground services. V30 fired against empty shipping_service on fresh deploys and the UPS Ground row later synced in with the default TRUE. Now flipped.</t>
         </is>
       </c>
       <c r="AC90" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -16838,12 +16844,13 @@
       <c r="AA111" s="15" t="n"/>
       <c r="AB111" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (a601e4aa): Custom Fields page says "Client scope" / "Platform-wide (all clients)"; description scrubbed.</t>
+          <t>Fixed on dev (a601e4aa): Custom Fields page says "Client scope" / "Platform-wide (all clients)"; description scrubbed.
+R6+1 (e17bf946, 2026-10-15): Tenant→client wording on CustomFieldsSection, PrintersPage scanner enroll, InvoiceCopiesMatrix, LabelTemplateEditorPage, LabelTemplatesListPage, OutputDestinationsPage doc / dest type dropdowns (humanised codes).</t>
         </is>
       </c>
       <c r="AC111" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -17926,12 +17933,13 @@
       <c r="AA119" s="15" t="n"/>
       <c r="AB119" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (9681f4ff): Output Destinations IAE now 400; create still fails on missing config - needs service-side fix later.</t>
+          <t>Fixed on dev (9681f4ff): Output Destinations IAE now 400; create still fails on missing config - needs service-side fix later.
+R6+1 (afeb4111, 2026-10-15): @JdbcTypeCode(SqlTypes.JSON) on ClientOutputDestination.config. Hibernate 6 was binding the String field as VARCHAR and Postgres rejected every save with 'column is of type jsonb but expression is of type character varying' → 500 on every destination create. Create now persists cleanly.</t>
         </is>
       </c>
       <c r="AC119" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -18067,12 +18075,13 @@
       <c r="AA120" s="15" t="n"/>
       <c r="AB120" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (9681f4ff): formatDateTime treats Z-less timestamps as UTC so IST operators see wall-clock time.</t>
+          <t>Fixed on dev (9681f4ff): formatDateTime treats Z-less timestamps as UTC so IST operators see wall-clock time.
+R6+1 (e17bf946, 2026-10-15): NotificationTemplatesPage 'Updated' line now routes through formatDateTime (treats Z-less backend timestamps as UTC).</t>
         </is>
       </c>
       <c r="AC120" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -18341,12 +18350,13 @@
       <c r="AA122" s="15" t="n"/>
       <c r="AB122" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (V158 6754690c): V158 deletes orphan tenant_settings rows (MKL274 removed).</t>
+          <t>Fixed on dev (V158 6754690c): V158 deletes orphan tenant_settings rows (MKL274 removed).
+R6+1 (afeb4111, 2026-10-15): PUT /external-systems/{id}/tenant-routings/{tenantCode} now 400s on an unknown client code so a FE typo can't seed a new orphan after V158's retroactive cleanup.</t>
         </is>
       </c>
       <c r="AC122" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -18873,12 +18883,13 @@
       <c r="AA126" s="15" t="n"/>
       <c r="AB126" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (d24684cc): Currencies description no longer references a non-existent per-tenant allowlist.</t>
+          <t>Fixed on dev (d24684cc): Currencies description no longer references a non-existent per-tenant allowlist.
+R6+1 (e17bf946, 2026-10-15): CURRENCY_ALLOWLIST (15 currencies) in utils/money.ts drives Orders/New, Customs profile, Client Identity + Markup. MXN / NZD / BRL etc. that were a client default but not pickable on the order form are now consistent across all three screens.</t>
         </is>
       </c>
       <c r="AC126" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -20070,12 +20081,13 @@
       <c r="AA135" s="15" t="n"/>
       <c r="AB135" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (a601e4aa): Writeback Journal Status cell humanises; Retry hidden on OK rows.</t>
+          <t>Fixed on dev (a601e4aa): Writeback Journal Status cell humanises; Retry hidden on OK rows.
+R6+1 (e17bf946, 2026-10-15): SKIPPED_INACTIVE added to the WritebackJournalStatus union + badge map so the humanised cell doesn't rely on a hard cast.</t>
         </is>
       </c>
       <c r="AC135" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(audit): R6+1 test-suite catch-up notes
Appends a one-line note on 7 bug rows (BUG-022/029/057/061/109/118/138)
pointing at today's test-fix commits (8cb8b4ba + 46d6db84). Most are
pure test lock-in; BUG-118's entry also documents a latent SERA
Idempotency-Key v3→v4 bug caught by the test rebuild and fixed in
8cb8b4ba.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -5135,7 +5135,8 @@
       <c r="AB23" s="15" t="inlineStr">
         <is>
           <t>Fixed on dev (a601e4aa): Delivery log recipient filter now escapes % _ and query uses ESCAPE "\\".
-R6+1 (afeb4111+e17bf946, 2026-10-15): Spread ESCAPE '\' + escapeLike() to WarehouseRepository, AdminUserService (Criteria API) and AuditLogRepositoryCustomImpl. Delivery-log fix (a601e4aa) now matches every other search path.</t>
+R6+1 (afeb4111+e17bf946, 2026-10-15): Spread ESCAPE '\' + escapeLike() to WarehouseRepository, AdminUserService (Criteria API) and AuditLogRepositoryCustomImpl. Delivery-log fix (a601e4aa) now matches every other search path.
+Test fix (46d6db84, 2026-10-15): — no code change, just test lock-in.</t>
         </is>
       </c>
       <c r="AC23" s="15" t="inlineStr">
@@ -6066,7 +6067,8 @@
       <c r="AA30" s="15" t="n"/>
       <c r="AB30" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (3a9a749e): DHL/FEDEX account input strips non-digits onChange + inputMode=numeric so the field physically cannot hold letters.</t>
+          <t>Fixed on dev (3a9a749e): DHL/FEDEX account input strips non-digits onChange + inputMode=numeric so the field physically cannot hold letters.
+Test fix (46d6db84, 2026-10-15): tests now assert UPS maxLength 10 + DHL maxLength 12 to match the 6-10 / 9-12 widening.</t>
         </is>
       </c>
       <c r="AC30" s="15" t="inlineStr">
@@ -9722,7 +9724,8 @@
       <c r="AA58" s="15" t="n"/>
       <c r="AB58" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (839f1ef8): FEDEX order form + per-carrier editor modals now read labelFormatsForCarrier() (DB registry); FEDEX added to the bootstrap list to mirror V120 seed.</t>
+          <t>Fixed on dev (839f1ef8): FEDEX order form + per-carrier editor modals now read labelFormatsForCarrier() (DB registry); FEDEX added to the bootstrap list to mirror V120 seed.
+Test fix (46d6db84, 2026-10-15): — no code change, just test lock-in.</t>
         </is>
       </c>
       <c r="AC58" s="15" t="inlineStr">
@@ -10264,7 +10267,8 @@
       <c r="AB62" s="15" t="inlineStr">
         <is>
           <t>Fixed on dev (cb9e4ed5): SystemChannelSection scrubbed TENANT_CHANNEL_NOT_ENABLED raw code; "tenant" -&gt; "client".
-R6+1 (afeb4111+e17bf946, 2026-10-15): Scrubbed internal copy on SystemSettings specs (backend), workspaceRoutes descriptions, Carrier Accounts, Code Maps, Cutoffs &amp; Holidays, External Systems, SystemSettingsPage deployment banner, DTC Scheduler 'Last changed by V&lt;n&gt;', Carrier Limits resolver blurb.</t>
+R6+1 (afeb4111+e17bf946, 2026-10-15): Scrubbed internal copy on SystemSettings specs (backend), workspaceRoutes descriptions, Carrier Accounts, Code Maps, Cutoffs &amp; Holidays, External Systems, SystemSettingsPage deployment banner, DTC Scheduler 'Last changed by V&lt;n&gt;', Carrier Limits resolver blurb.
+Test fix (46d6db84, 2026-10-15): SystemChannelSection test no longer asserts the scrubbed raw TENANT_CHANNEL_NOT_ENABLED code is rendered.</t>
         </is>
       </c>
       <c r="AC62" s="15" t="inlineStr">
@@ -16704,7 +16708,8 @@
       <c r="AA110" s="15" t="n"/>
       <c r="AB110" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (0fad4a45): Added renderWithTemplate(orderNo, templateId); controller ?templateId query param; FE passes previewContext.id so Preview renders THIS template.</t>
+          <t>Fixed on dev (0fad4a45): Added renderWithTemplate(orderNo, templateId); controller ?templateId query param; FE passes previewContext.id so Preview renders THIS template.
+Test fix (46d6db84, 2026-10-15): fetchPreviewObjectUrl now asserts the second-arg template id (previewContext.id) that landed with 0fad4a45.</t>
         </is>
       </c>
       <c r="AC110" s="15" t="inlineStr">
@@ -17934,7 +17939,8 @@
       <c r="AB119" s="15" t="inlineStr">
         <is>
           <t>Fixed on dev (9681f4ff): Output Destinations IAE now 400; create still fails on missing config - needs service-side fix later.
-R6+1 (afeb4111, 2026-10-15): @JdbcTypeCode(SqlTypes.JSON) on ClientOutputDestination.config. Hibernate 6 was binding the String field as VARCHAR and Postgres rejected every save with 'column is of type jsonb but expression is of type character varying' → 500 on every destination create. Create now persists cleanly.</t>
+R6+1 (afeb4111, 2026-10-15): @JdbcTypeCode(SqlTypes.JSON) on ClientOutputDestination.config. Hibernate 6 was binding the String field as VARCHAR and Postgres rejected every save with 'column is of type jsonb but expression is of type character varying' → 500 on every destination create. Create now persists cleanly.
+Test-suite fix (8cb8b4ba, 2026-10-15): also caught a latent bug — forStampsTopup returned a v3 UUID (nameUUIDFromBytes), which SERA rejects with error 800001 'Idempotency-Key invalid'. Topup now routes through stampsKey() like every other forStamps* helper so the version bits are stamped v4. Backfilled test: IdempotencyKeysStampsSeraTest.everyStampsKeyIsAStableV4Uuid.</t>
         </is>
       </c>
       <c r="AC119" s="15" t="inlineStr">
@@ -20625,7 +20631,8 @@
       <c r="AA139" s="15" t="n"/>
       <c r="AB139" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (a8af5b2a): carriersStepComplete requires every staged draft to carry non-blank clientId AND clientSecret.</t>
+          <t>Fixed on dev (a8af5b2a): carriersStepComplete requires every staged draft to carry non-blank clientId AND clientSecret.
+Test fix (46d6db84, 2026-10-15): importer-broker fixture now seeds non-blank clientId+clientSecret so the carriersStepComplete guard lets Submit through.</t>
         </is>
       </c>
       <c r="AC139" s="15" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): final R6+1 pass — 41 pending bugs → 0
- 4 bugs got net-new code today (BUG-076/079/099/130) via 2207535b
  + 0b501583. Each gets a tracker note pointing at the commit.
- 37 bugs were already-landed-on-HEAD per the dev commits log; a
  Explore-agent sweep confirmed each fix is physically in the file.
  Marked Fixed-in-build=2026-10-15 so the R7 tester has one clean
  retest batch instead of chasing the 2026-10-14 tracker rows.

All 53 R6 pending bugs are now either Fixed (49) or Deferred (4) with
today's build date. Zero bugs show Dev-status=Fixed with a stale
Fixed-in-build date.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -4627,7 +4627,7 @@
       </c>
       <c r="AC19" s="15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="AC30" s="15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="AC37" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="AC39" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -9730,7 +9730,7 @@
       </c>
       <c r="AC58" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -12250,12 +12250,13 @@
       <c r="AA77" s="15" t="n"/>
       <c r="AB77" s="15" t="inlineStr">
         <is>
-          <t>Fix landed earlier this session: CSV formula-injection guard shipped as 45c6b922 earlier.</t>
+          <t>Fix landed earlier this session: CSV formula-injection guard shipped as 45c6b922 earlier.
+R6+1 (0b501583, 2026-10-15): FE csv.ts csvCell now prefixes '=/+/-/@/TAB' with a single quote (mirrors backend).</t>
         </is>
       </c>
       <c r="AC77" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -12389,7 +12390,7 @@
       </c>
       <c r="AC78" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -12523,7 +12524,7 @@
       </c>
       <c r="AC79" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -12657,12 +12658,13 @@
       <c r="AA80" s="15" t="n"/>
       <c r="AB80" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (6754690c): Warehouse State input forces uppercase on change.</t>
+          <t>Fixed on dev (6754690c): Warehouse State input forces uppercase on change.
+R6+1 (2207535b, 2026-10-15): Warehouses grid upper-cases state at render too; legacy 'il' rows now display 'IL' without a resave.</t>
         </is>
       </c>
       <c r="AC80" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -12804,7 +12806,7 @@
       </c>
       <c r="AC81" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -13074,7 +13076,7 @@
       </c>
       <c r="AC83" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -14683,7 +14685,7 @@
       </c>
       <c r="AC95" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -14820,7 +14822,7 @@
       </c>
       <c r="AC96" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -14957,7 +14959,7 @@
       </c>
       <c r="AC97" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -15230,7 +15232,7 @@
       </c>
       <c r="AC99" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -15362,12 +15364,13 @@
       <c r="AA100" s="15" t="n"/>
       <c r="AB100" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (9681f4ff): Field marking still TODO but 500 is now 400 "references something that doesn't exist".</t>
+          <t>Fixed on dev (9681f4ff): Field marking still TODO but 500 is now 400 "references something that doesn't exist".
+R6+1 (2207535b, 2026-10-15): CutoffAdminController pre-validates warehouseId FK + throws IAE naming the field.</t>
         </is>
       </c>
       <c r="AC100" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -15633,7 +15636,7 @@
       </c>
       <c r="AC102" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -15764,7 +15767,7 @@
       </c>
       <c r="AC103" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -15902,7 +15905,7 @@
       </c>
       <c r="AC104" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -16040,7 +16043,7 @@
       </c>
       <c r="AC105" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -16313,7 +16316,7 @@
       </c>
       <c r="AC107" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -16714,7 +16717,7 @@
       </c>
       <c r="AC110" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -16992,7 +16995,7 @@
       </c>
       <c r="AC112" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -17129,7 +17132,7 @@
       </c>
       <c r="AC113" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -17395,7 +17398,7 @@
       </c>
       <c r="AC115" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -17532,7 +17535,7 @@
       </c>
       <c r="AC116" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -17669,7 +17672,7 @@
       </c>
       <c r="AC117" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -17806,7 +17809,7 @@
       </c>
       <c r="AC118" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -18224,7 +18227,7 @@
       </c>
       <c r="AC121" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -18757,7 +18760,7 @@
       </c>
       <c r="AC125" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -19559,12 +19562,13 @@
       <c r="AA131" s="15" t="n"/>
       <c r="AB131" s="15" t="inlineStr">
         <is>
-          <t>Fixed on dev (V157): V157 redacts client_id in old carrier_api_log rows.</t>
+          <t>Fixed on dev (V157): V157 redacts client_id in old carrier_api_log rows.
+R6+1 (V162 2207535b, 2026-10-15): V162 masks client_id at START of carrier_api_log request_body; V157's regex only caught `?`/`&amp;` prefixes, FedEx form bodies open with the field.</t>
         </is>
       </c>
       <c r="AC131" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -20230,7 +20234,7 @@
       </c>
       <c r="AC136" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -20637,7 +20641,7 @@
       </c>
       <c r="AC139" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -20774,7 +20778,7 @@
       </c>
       <c r="AC140" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -20916,7 +20920,7 @@
       </c>
       <c r="AC141" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -21308,7 +21312,7 @@
       </c>
       <c r="AC144" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -21441,7 +21445,7 @@
       </c>
       <c r="AC145" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -21574,7 +21578,7 @@
       </c>
       <c r="AC146" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -21708,7 +21712,7 @@
       </c>
       <c r="AC147" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -21842,7 +21846,7 @@
       </c>
       <c r="AC148" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -21975,7 +21979,7 @@
       </c>
       <c r="AC149" s="15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(audit): add R6+1 wrap-up note on Summary sheet
Summary row 18 records the 2026-10-15 follow-up pass:
 - 16 R6+1 code fixes shipped (12 earlier + 4 follow-ups)
 - 37 bugs verified on HEAD + marked Fixed-in-build=2026-10-15
 - 1 latent SERA Idempotency-Key bug caught + fixed
 - full test suites green (backend 4108/0, FE 1065/0/12-skip)
 - HEAD at commit 5f1d0e52

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -689,6 +689,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -916,6 +917,18 @@
       <c r="E17" s="20" t="n"/>
       <c r="F17" s="20" t="n"/>
       <c r="G17" s="21" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>R6+1 wrap-up</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-15 — follow-up on all 53 R6-pending bugs. 4 net-new code fixes shipped today (BUG-076/079/099/130 via 2207535b + 0b501583); 12 R6+1 code fixes shipped earlier the same day (BUG-022/046/061/075/087/089/110/118/119/121/125/134 via afeb4111 + e17bf946); 37 bugs verified fixed on HEAD per earlier dev commits and marked Fixed-in-build=2026-10-15. One latent SERA Idempotency-Key v3→v4 bug (forStampsTopup) also caught by the test-suite rebuild and fixed in 8cb8b4ba. Full suites green: backend 4108/0, frontend 1065/0/12-skip. HEAD at commit 5f1d0e52.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): pull 9 Deferred bugs forward to Fixed on R6+1 pass
Today's sweep confirmed 7 bugs already on HEAD per earlier dev
commits (BUG-068/072/073/081/105/107/127) + 2 net-new code fixes
(BUG-092/093 via 3508b210). All 9 flipped Dev=Fixed with today's
Fixed-in-build.

Deferred count: 23 → 14. BUG-147 was already Fixed in prior pass;
remaining 14 Deferred still carry the dev's 'needs ... next round'
notes (BUG-007/017/070/085/086/088/090/097/123/128/129/131/136/137).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -689,7 +689,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -11202,16 +11201,21 @@
       </c>
       <c r="Z69" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA69" s="15" t="n"/>
       <c r="AB69" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Unknown-route catchall lands on /dashboard but preserves nothing. Needs a NotFound page.</t>
-        </is>
-      </c>
-      <c r="AC69" s="15" t="n"/>
+          <t>Deferred to next round: Unknown-route catchall lands on /dashboard but preserves nothing. Needs a NotFound page.
+R6+1 (2026-10-15): Already on HEAD — in-shell NotFoundPage mounted at Route path='*' preserves the attempted URL.</t>
+        </is>
+      </c>
+      <c r="AC69" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -11715,16 +11719,21 @@
       </c>
       <c r="Z73" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA73" s="15" t="n"/>
       <c r="AB73" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: FTR exemption passes without ITN on FedEx-to-Canada. Needs validation when exemption=None (using AES).</t>
-        </is>
-      </c>
-      <c r="AC73" s="15" t="n"/>
+          <t>Deferred to next round: FTR exemption passes without ITN on FedEx-to-Canada. Needs validation when exemption=None (using AES).
+R6+1 (2026-10-15): Already on HEAD — NewShipmentPage requires FTR exemption or AES ITN for US → CA shipments.</t>
+        </is>
+      </c>
+      <c r="AC73" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -11845,16 +11854,21 @@
       </c>
       <c r="Z74" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA74" s="15" t="n"/>
       <c r="AB74" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Price-&amp;-delivery box renders raw q.message; needs cleaner pass similar to validationChecklist.</t>
-        </is>
-      </c>
-      <c r="AC74" s="15" t="n"/>
+          <t>Deferred to next round: Price-&amp;-delivery box renders raw q.message; needs cleaner pass similar to validationChecklist.
+R6+1 (2026-10-15): Already on HEAD — ValidationQuote strips 'No price:' prefix and HTTP 5xx tail from quote.message.</t>
+        </is>
+      </c>
+      <c r="AC74" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
@@ -12945,16 +12959,21 @@
       </c>
       <c r="Z82" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA82" s="15" t="n"/>
       <c r="AB82" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Warehouse verify "VERIFICATION NOT SUPPORTED FOR THIS COUNTRY" when real reason is missing credentials. Wording.</t>
-        </is>
-      </c>
-      <c r="AC82" s="15" t="n"/>
+          <t>Deferred to next round: Warehouse verify "VERIFICATION NOT SUPPORTED FOR THIS COUNTRY" when real reason is missing credentials. Wording.
+R6+1 (2026-10-15): Already on HEAD — WarehouseEditorModal branches on credsMissing so the status reads 'Carrier credentials not configured'.</t>
+        </is>
+      </c>
+      <c r="AC82" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
@@ -14421,16 +14440,21 @@
       </c>
       <c r="Z93" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA93" s="15" t="n"/>
       <c r="AB93" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: tare &gt; max weight guard; needs save validation on Add Package.</t>
-        </is>
-      </c>
-      <c r="AC93" s="15" t="n"/>
+          <t>Deferred to next round: tare &gt; max weight guard; needs save validation on Add Package.
+R6+1 (3508b210, 2026-10-15): ShippingConfigService.savePreset now refuses tareWeight &gt; maxWeight at 422.</t>
+        </is>
+      </c>
+      <c r="AC93" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -14554,16 +14578,21 @@
       </c>
       <c r="Z94" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA94" s="15" t="n"/>
       <c r="AB94" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Duplicate alias silent replace; needs "updated existing" message in service.</t>
-        </is>
-      </c>
-      <c r="AC94" s="15" t="n"/>
+          <t>Deferred to next round: Duplicate alias silent replace; needs "updated existing" message in service.
+R6+1 (3508b210, 2026-10-15): upsertShipvia reports 'already existed — the existing mapping was updated' when the (clientCode, erpCode, dest*) row was pre-existing.</t>
+        </is>
+      </c>
+      <c r="AC94" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
@@ -16182,16 +16211,21 @@
       </c>
       <c r="Z106" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA106" s="15" t="n"/>
       <c r="AB106" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Importer search by country name/city; backend search needs expand.</t>
-        </is>
-      </c>
-      <c r="AC106" s="15" t="n"/>
+          <t>Deferred to next round: Importer search by country name/city; backend search needs expand.
+R6+1 (2026-10-15): Already on HEAD — ClientCustomsProfileServiceImpl.matchesSearch appends full country name to the needle so 'canada' / 'mexico' etc. hit.</t>
+        </is>
+      </c>
+      <c r="AC106" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
@@ -16456,16 +16490,21 @@
       </c>
       <c r="Z108" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA108" s="15" t="n"/>
       <c r="AB108" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Logo content magic-byte check; current fix is MIME-level only.</t>
-        </is>
-      </c>
-      <c r="AC108" s="15" t="n"/>
+          <t>Deferred to next round: Logo content magic-byte check; current fix is MIME-level only.
+R6+1 (2026-10-15): Already on HEAD — LabelTemplateEditorPage.chooseLogo verifies PNG/JPEG magic bytes after the MIME check.</t>
+        </is>
+      </c>
+      <c r="AC108" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
@@ -19166,16 +19205,21 @@
       </c>
       <c r="Z128" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA128" s="15" t="n"/>
       <c r="AB128" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Export button (visible page) vs Export CSV (full) wording clarified later.</t>
-        </is>
-      </c>
-      <c r="AC128" s="15" t="n"/>
+          <t>Deferred to next round: Export button (visible page) vs Export CSV (full) wording clarified later.
+R6+1 (2026-10-15): Already on HEAD — AuditLogPage labels the second button 'Export all (CSV)' (full set) vs the AdvancedDataTable 'Export' (current page).</t>
+        </is>
+      </c>
+      <c r="AC128" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): BUG-128 flipped to Fixed (sprints 1 + 2 cover every named service)
After f14bcf08, every Settings surface the R6 tester called out for
BUG-128 writes to audit_log. Dev status flipped Fixed, Fixed-in-build
2026-10-15.

Deferred count: 14 -> 13.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -19347,17 +19347,22 @@
       </c>
       <c r="Z129" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA129" s="15" t="n"/>
       <c r="AB129" s="15" t="inlineStr">
         <is>
           <t>Deferred to next round: Big — audit calls on templates / code maps / customs profiles / custom fields / printers / scanners / mail. Multi-service pass.
-R6+1 sprint 1 (f46b6f01, 2026-10-15): AuditService wired into LabelTemplateServiceImpl, ClientCodeMapServiceImpl, ClientCustomsProfileServiceImpl, CustomFieldServiceImpl, ClientBillingMarkupServiceImpl, RoutingRuleServiceImpl, PrinterScanService + MailConfigService. 56/56 related unit tests green. Dev status stays Deferred because the second half (Printers CRUD / Cutoffs / Address book / Pickups / Output Destinations) is batched for sprint 2.</t>
-        </is>
-      </c>
-      <c r="AC129" s="15" t="n"/>
+R6+1 sprint 1 (f46b6f01, 2026-10-15): AuditService wired into LabelTemplateServiceImpl, ClientCodeMapServiceImpl, ClientCustomsProfileServiceImpl, CustomFieldServiceImpl, ClientBillingMarkupServiceImpl, RoutingRuleServiceImpl, PrinterScanService + MailConfigService. 56/56 related unit tests green. Dev status stays Deferred because the second half (Printers CRUD / Cutoffs / Address book / Pickups / Output Destinations) is batched for sprint 2.
+R6+1 sprint 2 (f14bcf08, 2026-10-15): AuditService wired into PrinterService (Settings &gt; Printers CRUD), CutoffAdminController (cutoff rules + holidays), SavedRecipientServiceImpl (Address book) and OutputDestinationAdminService (output destinations). Pickups already recorded via CarrierEodLogger. 38/38 related unit tests green.</t>
+        </is>
+      </c>
+      <c r="AC129" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): flip 3 more Deferred bugs Fixed
BUG-085 + BUG-086 already landed on HEAD; BUG-090 fixed today via
c96e743f. Deferred: 13 -> 10.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -13500,16 +13500,21 @@
       </c>
       <c r="Z86" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA86" s="15" t="n"/>
       <c r="AB86" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Audit entry for invite resend/revoke; needs recordAction wiring.</t>
-        </is>
-      </c>
-      <c r="AC86" s="15" t="n"/>
+          <t>Deferred to next round: Audit entry for invite resend/revoke; needs recordAction wiring.
+R6+1 (2026-10-15): Already on HEAD — AdminUserInviteController calls adminUserService.recordInviteResent / recordInviteRevoked which writes INVITE_RESENT / INVITE_REVOKED rows to user_admin_audit so Recent admin actions picks them up.</t>
+        </is>
+      </c>
+      <c r="AC86" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
@@ -13638,16 +13643,21 @@
       </c>
       <c r="Z87" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA87" s="15" t="n"/>
       <c r="AB87" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Mail form autofill unchanged; needs same new-password treatment as Carrier Accounts.</t>
-        </is>
-      </c>
-      <c r="AC87" s="15" t="n"/>
+          <t>Deferred to next round: Mail form autofill unchanged; needs same new-password treatment as Carrier Accounts.
+R6+1 (2026-10-15): Already on HEAD — MailProviderFormModal uses autoComplete='new-password' on every secret-typed field so Chrome stops dumping the Multiship sign-in into them.</t>
+        </is>
+      </c>
+      <c r="AC87" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -14181,16 +14191,21 @@
       </c>
       <c r="Z91" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA91" s="15" t="n"/>
       <c r="AB91" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Shipping Catalog tabs don't share origin. Needs lifted-state origin filter.</t>
-        </is>
-      </c>
-      <c r="AC91" s="15" t="n"/>
+          <t>Deferred to next round: Shipping Catalog tabs don't share origin. Needs lifted-state origin filter.
+R6+1 (2026-10-15): R6+1 (c96e743f, 2026-10-15): ShippingCatalogPage lifts origin + onOriginChange and passes to both ShippingServicesPage and PackagesPage, so the sub-tabs now share the filter the page description promised.</t>
+        </is>
+      </c>
+      <c r="AC91" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): BUG-129 + BUG-136 flipped Fixed
Deferred: 10 -> 8.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -19501,16 +19501,21 @@
       </c>
       <c r="Z130" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA130" s="15" t="n"/>
       <c r="AB130" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Logs filter Entity type + Action lists need DB-driven population.</t>
-        </is>
-      </c>
-      <c r="AC130" s="15" t="n"/>
+          <t>Deferred to next round: Logs filter Entity type + Action lists need DB-driven population.
+R6+1 (c39e9e6e, 2026-10-15): AuditLogPage dropdowns extended to cover every AuditService entity + action constant (IMPORT_BATCH + LABEL_REGENERATED / LABEL_VOID_REFUSED / CARRIER_REJECTED / IMPORT_SAVED / IMPORT_GENERATED / LOGIN_FAILED). Hardcoded against the backend constants rather than DB-driven - swap to a /api/v1/audit-log/filter-values endpoint if the enum ever grows.</t>
+        </is>
+      </c>
+      <c r="AC130" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
@@ -20438,16 +20443,21 @@
       </c>
       <c r="Z137" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA137" s="15" t="n"/>
       <c r="AB137" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: Return label origin same as recipient; needs ReturnFromCustomer prefill rewrite.</t>
-        </is>
-      </c>
-      <c r="AC137" s="15" t="n"/>
+          <t>Deferred to next round: Return label origin same as recipient; needs ReturnFromCustomer prefill rewrite.
+R6+1 (c39e9e6e, 2026-10-15): switching SHIPMENT -&gt; RETURN now clears the sender block when it still matches the warehouse address exactly, so 'Return from * customer' opens blank for the operator to fill. Anything typed is preserved.</t>
+        </is>
+      </c>
+      <c r="AC137" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(audit): BUG-123 partial fix note + BUG-137 flipped Fixed
BUG-123: CountrySelect keyboard support shipped via 8ab23db5. HS code
already shipped earlier. The broader dialog focus/escape audit stays
Deferred — that is a cross-cutting sweep across every Settings modal.

BUG-137: FedExConnector shipper block builds from request.getShipperXxx
verbatim; BUG-136 fix stops the FE from pre-filling the warehouse in
Return mode. Every NEW return label will carry the customer's address.
Historical stored ZPL for #934194 stays unchanged (immutable).

Deferred: 8 -> 7.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
+++ b/docs/audits/Multiship_Bug_List_2026-10-14_R6.xlsx
@@ -18693,10 +18693,15 @@
       <c r="AA124" s="15" t="n"/>
       <c r="AB124" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: HS lookup keyboard support + dialog focus/escape audit.</t>
-        </is>
-      </c>
-      <c r="AC124" s="15" t="n"/>
+          <t>Deferred to next round: HS lookup keyboard support + dialog focus/escape audit.
+R6+1 (8ab23db5, 2026-10-15): CountrySelect now carries ArrowDown/Up/Enter/Escape keyboard support + aria-activedescendant / role=combobox / role=option so the shared country picker is reachable from the keyboard. HS code combobox landed earlier. Broader dialog focus/escape audit stays Deferred - that is a cross-cutting sweep across every Settings modal.</t>
+        </is>
+      </c>
+      <c r="AC124" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
@@ -20581,16 +20586,21 @@
       </c>
       <c r="Z138" s="15" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="AA138" s="15" t="n"/>
       <c r="AB138" s="15" t="inlineStr">
         <is>
-          <t>Deferred to next round: ZPL return label SHIP FROM "Multiship Warehouse, Bengaluru"; return-shipper is wrong at label-generation time, baked into the stored ZPL. Needs FedExConnector return branch fix. User chose deep-dive.</t>
-        </is>
-      </c>
-      <c r="AC138" s="15" t="n"/>
+          <t>Deferred to next round: ZPL return label SHIP FROM "Multiship Warehouse, Bengaluru"; return-shipper is wrong at label-generation time, baked into the stored ZPL. Needs FedExConnector return branch fix. User chose deep-dive.
+R6+1 (2026-10-15): FedExConnector builds the shipper block from request.getShipperXxx() verbatim - no tenant-settings fallback. BUG-136 fix (c39e9e6e) stops the FE from pre-filling the warehouse address in Return mode, so every NEW return label will carry the customer's address on SHIP FROM. Historical ZPL for #934194 remains unchanged (stored label is immutable).</t>
+        </is>
+      </c>
+      <c r="AC138" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">

</xml_diff>